<commit_message>
fix: planes de carrera canonicos curados, iconos perfeccionados, modal de descarga condicional, guia libros ironica, enlaces de becas y dashboard admin mobile
</commit_message>
<xml_diff>
--- a/data/mapas/Mapa_de_Carrera_Biologia.xlsx
+++ b/data/mapas/Mapa_de_Carrera_Biologia.xlsx
@@ -555,13 +555,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="J2" s="5" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="J3" s="5">
-        <f>COUNTIF(B6:B55, "SI")</f>
+        <f>COUNTIF(B6:B43, "SI")</f>
         <v/>
       </c>
     </row>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="J4" s="5">
-        <f>COUNTIF(C6:C55, "SI")</f>
+        <f>COUNTIF(C6:C43, "SI")</f>
         <v/>
       </c>
     </row>
@@ -667,14 +667,14 @@
         </is>
       </c>
       <c r="J5" s="5">
-        <f>COUNTIF(F6:F55, "ADEUDA FINAL")</f>
+        <f>COUNTIF(F6:F43, "ADEUDA FINAL")</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Pedagogía</t>
+          <t>Introducción a la Biología y Sistemas Vivientes</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
@@ -710,14 +710,14 @@
         </is>
       </c>
       <c r="J6" s="12">
-        <f>COUNTIF(B6:B55, "SI")/44</f>
+        <f>COUNTIF(B6:B43, "SI")/34</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Didáctica General</t>
+          <t>Biología Celular y Molecular</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
@@ -753,14 +753,14 @@
         </is>
       </c>
       <c r="J7" s="12">
-        <f>COUNTIF(C6:C55, "SI")/44</f>
+        <f>COUNTIF(C6:C43, "SI")/34</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Introducción a la Disciplina</t>
+          <t>Diversidad Vegetal I</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -794,7 +794,7 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Práctica Docente I</t>
+          <t>Química General e Inorgánica</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
@@ -831,10 +831,37 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>📌 2° AÑO</t>
-        </is>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Matemática y Estadística Aplicada</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>1° Año</t>
+        </is>
+      </c>
+      <c r="E10" s="10">
+        <f>IF(B10="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F10" s="10">
+        <f>IF(C10="SI", "APROBADO", IF(B10="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G10" s="11">
+        <f>IF(C10="SI", "🟢 Aprobada", IF(B10="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
@@ -845,7 +872,7 @@
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Psicología Educacional</t>
+          <t>Pedagogía</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -860,7 +887,7 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>2° Año</t>
+          <t>1° Año</t>
         </is>
       </c>
       <c r="E11" s="10">
@@ -884,7 +911,7 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Sociología de la Educación</t>
+          <t>Lectura, Escritura y Oralidad I (LEO 1)</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -899,7 +926,7 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>2° Año</t>
+          <t>1° Año</t>
         </is>
       </c>
       <c r="E12" s="10">
@@ -923,7 +950,7 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Sujetos de la Educación</t>
+          <t>Trabajo de Campo I</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
@@ -938,7 +965,7 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>2° Año</t>
+          <t>1° Año</t>
         </is>
       </c>
       <c r="E13" s="10">
@@ -960,49 +987,49 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Práctica Docente II</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>📌 2° AÑO</t>
+        </is>
+      </c>
+      <c r="I14" s="14" t="inlineStr">
+        <is>
+          <t>5. El panel lateral calcula tu avance y porcentaje de carrera en vivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Diversidad Vegetal II</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>2° Año</t>
         </is>
       </c>
-      <c r="E14" s="10">
-        <f>IF(B14="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F14" s="10">
-        <f>IF(C14="SI", "APROBADO", IF(B14="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G14" s="11">
-        <f>IF(C14="SI", "🟢 Aprobada", IF(B14="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
-      </c>
-      <c r="I14" s="14" t="inlineStr">
-        <is>
-          <t>5. El panel lateral calcula tu avance y porcentaje de carrera en vivo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>📌 3° AÑO</t>
-        </is>
+      <c r="E15" s="10">
+        <f>IF(B15="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F15" s="10">
+        <f>IF(C15="SI", "APROBADO", IF(B15="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G15" s="11">
+        <f>IF(C15="SI", "🟢 Aprobada", IF(B15="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -1013,7 +1040,7 @@
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Historia Social de la Educación</t>
+          <t>Diversidad Animal I (Invertebrados)</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
@@ -1028,7 +1055,7 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>3° Año</t>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E16" s="10">
@@ -1047,7 +1074,7 @@
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Residencia I</t>
+          <t>Anatomía y Fisiología Humana</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
@@ -1062,7 +1089,7 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>3° Año</t>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E17" s="10">
@@ -1081,7 +1108,7 @@
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Espacio de Definición Institucional</t>
+          <t>Química Orgánica y Biológica</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
@@ -1096,7 +1123,7 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>3° Año</t>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E18" s="10">
@@ -1115,7 +1142,7 @@
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Práctica Docente III</t>
+          <t>Didáctica General</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
@@ -1130,7 +1157,7 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>3° Año</t>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E19" s="10">
@@ -1146,17 +1173,44 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>📌 4° AÑO</t>
-        </is>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Psicología Educacional</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>2° Año</t>
+        </is>
+      </c>
+      <c r="E20" s="10">
+        <f>IF(B20="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F20" s="10">
+        <f>IF(C20="SI", "APROBADO", IF(B20="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G20" s="11">
+        <f>IF(C20="SI", "🟢 Aprobada", IF(B20="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Residencia II / Taller de Cierre</t>
+          <t>Sujetos de la Educación</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
@@ -1171,7 +1225,7 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>4° Año</t>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E21" s="10">
@@ -1190,7 +1244,7 @@
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>Ética y Trabajo Docente</t>
+          <t>Trabajo de Campo II</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
@@ -1205,7 +1259,7 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>4° Año</t>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E22" s="10">
@@ -1221,44 +1275,17 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>Investigación Educativa</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>4° Año</t>
-        </is>
-      </c>
-      <c r="E23" s="10">
-        <f>IF(B23="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F23" s="10">
-        <f>IF(C23="SI", "APROBADO", IF(B23="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G23" s="11">
-        <f>IF(C23="SI", "🟢 Aprobada", IF(B23="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>📌 3° AÑO</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>Práctica Docente IV</t>
+          <t>Diversidad Animal II (Vertebrados)</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
@@ -1273,7 +1300,7 @@
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>4° Año</t>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E24" s="10">
@@ -1289,17 +1316,44 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>📌 5° AÑO (NIVEL SUPERIOR / TRAMO SUPERIOR)</t>
-        </is>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Genética General y Molecular</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>3° Año</t>
+        </is>
+      </c>
+      <c r="E25" s="10">
+        <f>IF(B25="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F25" s="10">
+        <f>IF(C25="SI", "APROBADO", IF(B25="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G25" s="11">
+        <f>IF(C25="SI", "🟢 Aprobada", IF(B25="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>Seminario de Especialización Superior I</t>
+          <t>Ecología General y de Poblaciones</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
@@ -1314,7 +1368,7 @@
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>5° Año (Nivel Superior / Tramo Superior)</t>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E26" s="10">
@@ -1333,7 +1387,7 @@
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Taller de Investigación Aplicada</t>
+          <t>Didáctica de la Biología I</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
@@ -1348,7 +1402,7 @@
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>5° Año (Nivel Superior / Tramo Superior)</t>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E27" s="10">
@@ -1367,7 +1421,7 @@
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>Didáctica de Nivel Superior</t>
+          <t>Ciencias de la Tierra y Dinámica Terrestre</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
@@ -1382,7 +1436,7 @@
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>5° Año (Nivel Superior / Tramo Superior)</t>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E28" s="10">
@@ -1401,7 +1455,7 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Práctica de Nivel Superior I</t>
+          <t>Historia Social de la Educación</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
@@ -1416,7 +1470,7 @@
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>5° Año (Nivel Superior / Tramo Superior)</t>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E29" s="10">
@@ -1432,17 +1486,44 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>📌 6° AÑO (NIVEL SUPERIOR / TRAMO SUPERIOR)</t>
-        </is>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Derechos Humanos, Sociedad y Estado</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>3° Año</t>
+        </is>
+      </c>
+      <c r="E30" s="10">
+        <f>IF(B30="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F30" s="10">
+        <f>IF(C30="SI", "APROBADO", IF(B30="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G30" s="11">
+        <f>IF(C30="SI", "🟢 Aprobada", IF(B30="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Seminario de Especialización Superior II</t>
+          <t>Construcción de la Práctica Docente I</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -1457,7 +1538,7 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>6° Año (Nivel Superior / Tramo Superior)</t>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E31" s="10">
@@ -1473,44 +1554,17 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>Tesis / Trabajo Final de Licenciatura</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>6° Año (Nivel Superior / Tramo Superior)</t>
-        </is>
-      </c>
-      <c r="E32" s="10">
-        <f>IF(B32="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F32" s="10">
-        <f>IF(C32="SI", "APROBADO", IF(B32="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G32" s="11">
-        <f>IF(C32="SI", "🟢 Aprobada", IF(B32="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>📌 4° AÑO</t>
+        </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Práctica de Nivel Superior II</t>
+          <t>Evolución y Paleontología</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
@@ -1525,7 +1579,7 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>6° Año (Nivel Superior / Tramo Superior)</t>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E33" s="10">
@@ -1544,7 +1598,7 @@
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>Acreditación de Residencia Superior</t>
+          <t>Fisiología y Morfología Comparada</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
@@ -1559,7 +1613,7 @@
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>6° Año (Nivel Superior / Tramo Superior)</t>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E34" s="10">
@@ -1575,17 +1629,44 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>📌 GENERAL / OPTATIVAS</t>
-        </is>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Educación para la Salud y el Ambiente</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>4° Año</t>
+        </is>
+      </c>
+      <c r="E35" s="10">
+        <f>IF(B35="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F35" s="10">
+        <f>IF(C35="SI", "APROBADO", IF(B35="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G35" s="11">
+        <f>IF(C35="SI", "🟢 Aprobada", IF(B35="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>Aytp</t>
+          <t>Didáctica de la Biología II</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
@@ -1600,7 +1681,7 @@
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>General / Optativas</t>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E36" s="10">
@@ -1619,7 +1700,7 @@
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>Biodiversidad de las Plantas</t>
+          <t>Educación Sexual Integral (ESI)</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
@@ -1634,7 +1715,7 @@
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>General / Optativas</t>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E37" s="10">
@@ -1653,7 +1734,7 @@
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>Biología DE LAS PLANTAS II</t>
+          <t>Ética y Trabajo Docente</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
@@ -1668,7 +1749,7 @@
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>General / Optativas</t>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E38" s="10">
@@ -1687,7 +1768,7 @@
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>Biología DE LOS ANIMALES I</t>
+          <t>Residencia y Construcción de la Práctica Docente II</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
@@ -1702,7 +1783,7 @@
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>General / Optativas</t>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E39" s="10">
@@ -1718,44 +1799,17 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="8" t="inlineStr">
-        <is>
-          <t>Biología DE LOS ANIMALES III</t>
-        </is>
-      </c>
-      <c r="B40" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D40" s="10" t="inlineStr">
-        <is>
-          <t>General / Optativas</t>
-        </is>
-      </c>
-      <c r="E40" s="10">
-        <f>IF(B40="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F40" s="10">
-        <f>IF(C40="SI", "APROBADO", IF(B40="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G40" s="11">
-        <f>IF(C40="SI", "🟢 Aprobada", IF(B40="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>📌 TRAMO SUPERIOR / SEMINARIOS</t>
+        </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>Biología DE LOS MICROORGANISMOS</t>
+          <t>Seminario de Biotecnología y Sociedad</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
@@ -1770,7 +1824,7 @@
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>General / Optativas</t>
+          <t>Tramo Superior / Seminarios</t>
         </is>
       </c>
       <c r="E41" s="10">
@@ -1789,7 +1843,7 @@
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>Biología HUMANA I</t>
+          <t>Seminario de Epistemología de la Biología</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
@@ -1804,7 +1858,7 @@
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>General / Optativas</t>
+          <t>Tramo Superior / Seminarios</t>
         </is>
       </c>
       <c r="E42" s="10">
@@ -1823,7 +1877,7 @@
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>Biología MOLECULAR Y CELULAR</t>
+          <t>Taller de Investigación en Ciencias Naturales</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
@@ -1838,7 +1892,7 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>General / Optativas</t>
+          <t>Tramo Superior / Seminarios</t>
         </is>
       </c>
       <c r="E43" s="10">
@@ -1854,436 +1908,26 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t>Ciencias DE LA TIERRA</t>
-        </is>
-      </c>
-      <c r="B44" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C44" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D44" s="10" t="inlineStr">
-        <is>
-          <t>General / Optativas</t>
-        </is>
-      </c>
-      <c r="E44" s="10">
-        <f>IF(B44="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F44" s="10">
-        <f>IF(C44="SI", "APROBADO", IF(B44="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G44" s="11">
-        <f>IF(C44="SI", "🟢 Aprobada", IF(B44="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
-          <t>Didáctica. DE Educación EN EL AMBIENTE</t>
-        </is>
-      </c>
-      <c r="B45" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D45" s="10" t="inlineStr">
-        <is>
-          <t>General / Optativas</t>
-        </is>
-      </c>
-      <c r="E45" s="10">
-        <f>IF(B45="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F45" s="10">
-        <f>IF(C45="SI", "APROBADO", IF(B45="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G45" s="11">
-        <f>IF(C45="SI", "🟢 Aprobada", IF(B45="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>Dinamica Terrestre</t>
-        </is>
-      </c>
-      <c r="B46" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D46" s="10" t="inlineStr">
-        <is>
-          <t>General / Optativas</t>
-        </is>
-      </c>
-      <c r="E46" s="10">
-        <f>IF(B46="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F46" s="10">
-        <f>IF(C46="SI", "APROBADO", IF(B46="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G46" s="11">
-        <f>IF(C46="SI", "🟢 Aprobada", IF(B46="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t>Evolucion e Historia de Vida</t>
-        </is>
-      </c>
-      <c r="B47" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D47" s="10" t="inlineStr">
-        <is>
-          <t>General / Optativas</t>
-        </is>
-      </c>
-      <c r="E47" s="10">
-        <f>IF(B47="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F47" s="10">
-        <f>IF(C47="SI", "APROBADO", IF(B47="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G47" s="11">
-        <f>IF(C47="SI", "🟢 Aprobada", IF(B47="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="8" t="inlineStr">
-        <is>
-          <t>Física</t>
-        </is>
-      </c>
-      <c r="B48" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D48" s="10" t="inlineStr">
-        <is>
-          <t>General / Optativas</t>
-        </is>
-      </c>
-      <c r="E48" s="10">
-        <f>IF(B48="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F48" s="10">
-        <f>IF(C48="SI", "APROBADO", IF(B48="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G48" s="11">
-        <f>IF(C48="SI", "🟢 Aprobada", IF(B48="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="8" t="inlineStr">
-        <is>
-          <t>HISTORIA DE LA Educación ARGENTINA</t>
-        </is>
-      </c>
-      <c r="B49" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D49" s="10" t="inlineStr">
-        <is>
-          <t>General / Optativas</t>
-        </is>
-      </c>
-      <c r="E49" s="10">
-        <f>IF(B49="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F49" s="10">
-        <f>IF(C49="SI", "APROBADO", IF(B49="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G49" s="11">
-        <f>IF(C49="SI", "🟢 Aprobada", IF(B49="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t>Introduccion a los Sist. Vivientes</t>
-        </is>
-      </c>
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C50" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D50" s="10" t="inlineStr">
-        <is>
-          <t>General / Optativas</t>
-        </is>
-      </c>
-      <c r="E50" s="10">
-        <f>IF(B50="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F50" s="10">
-        <f>IF(C50="SI", "APROBADO", IF(B50="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G50" s="11">
-        <f>IF(C50="SI", "🟢 Aprobada", IF(B50="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="8" t="inlineStr">
-        <is>
-          <t>Matemática</t>
-        </is>
-      </c>
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D51" s="10" t="inlineStr">
-        <is>
-          <t>General / Optativas</t>
-        </is>
-      </c>
-      <c r="E51" s="10">
-        <f>IF(B51="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F51" s="10">
-        <f>IF(C51="SI", "APROBADO", IF(B51="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G51" s="11">
-        <f>IF(C51="SI", "🟢 Aprobada", IF(B51="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="8" t="inlineStr">
-        <is>
-          <t>Morfofisiología Comparada DE LOS ANIMALES y Ambiente</t>
-        </is>
-      </c>
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D52" s="10" t="inlineStr">
-        <is>
-          <t>General / Optativas</t>
-        </is>
-      </c>
-      <c r="E52" s="10">
-        <f>IF(B52="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F52" s="10">
-        <f>IF(C52="SI", "APROBADO", IF(B52="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G52" s="11">
-        <f>IF(C52="SI", "🟢 Aprobada", IF(B52="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="8" t="inlineStr">
-        <is>
-          <t>Psicología DEL DESARROLLO Y APREND</t>
-        </is>
-      </c>
-      <c r="B53" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D53" s="10" t="inlineStr">
-        <is>
-          <t>General / Optativas</t>
-        </is>
-      </c>
-      <c r="E53" s="10">
-        <f>IF(B53="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F53" s="10">
-        <f>IF(C53="SI", "APROBADO", IF(B53="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G53" s="11">
-        <f>IF(C53="SI", "🟢 Aprobada", IF(B53="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="8" t="inlineStr">
-        <is>
-          <t>Química</t>
-        </is>
-      </c>
-      <c r="B54" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C54" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D54" s="10" t="inlineStr">
-        <is>
-          <t>General / Optativas</t>
-        </is>
-      </c>
-      <c r="E54" s="10">
-        <f>IF(B54="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F54" s="10">
-        <f>IF(C54="SI", "APROBADO", IF(B54="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G54" s="11">
-        <f>IF(C54="SI", "🟢 Aprobada", IF(B54="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="8" t="inlineStr">
-        <is>
-          <t>Trabajo de Campo I</t>
-        </is>
-      </c>
-      <c r="B55" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C55" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D55" s="10" t="inlineStr">
-        <is>
-          <t>General / Optativas</t>
-        </is>
-      </c>
-      <c r="E55" s="10">
-        <f>IF(B55="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F55" s="10">
-        <f>IF(C55="SI", "APROBADO", IF(B55="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G55" s="11">
-        <f>IF(C55="SI", "🟢 Aprobada", IF(B55="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="I14:J14"/>
+  <mergeCells count="15">
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A14:G14"/>
     <mergeCell ref="I12:J12"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A40:G40"/>
     <mergeCell ref="I15:J15"/>
     <mergeCell ref="I10:J10"/>
-    <mergeCell ref="A35:G35"/>
     <mergeCell ref="I1:K1"/>
     <mergeCell ref="I11:J11"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A30:G30"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A15:G15"/>
     <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="I14:J14"/>
     <mergeCell ref="I9:J9"/>
-    <mergeCell ref="A10:G10"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B6 B7 B8 B9 B11 B12 B13 B14 B16 B17 B18 B19 B21 B22 B23 B24 B26 B27 B28 B29 B31 B32 B33 B34 B36 B37 B38 B39 B40 B41 B42 B43 B44 B45 B46 B47 B48 B49 B50 B51 B52 B53 B54 B55 C6 C7 C8 C9 C11 C12 C13 C14 C16 C17 C18 C19 C21 C22 C23 C24 C26 C27 C28 C29 C31 C32 C33 C34 C36 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Opción inválida" error="Por favor, elegí 'SI' o 'NO' de la lista desplegable." type="list">
+    <dataValidation sqref="B6 B7 B8 B9 B10 B11 B12 B13 B15 B16 B17 B18 B19 B20 B21 B22 B24 B25 B26 B27 B28 B29 B30 B31 B33 B34 B35 B36 B37 B38 B39 B41 B42 B43 C6 C7 C8 C9 C10 C11 C12 C13 C15 C16 C17 C18 C19 C20 C21 C22 C24 C25 C26 C27 C28 C29 C30 C31 C33 C34 C35 C36 C37 C38 C39 C41 C42 C43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Opción inválida" error="Por favor, elegí 'SI' o 'NO' de la lista desplegable." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: sincronizacion directa de los 18 correlativators de Drive, atomo de fisica, torre de pisa, calculadora minimalista, limite y enumeracion de suscriptores, y dashboard analitico con selector de periodo
</commit_message>
<xml_diff>
--- a/data/mapas/Mapa_de_Carrera_Biologia.xlsx
+++ b/data/mapas/Mapa_de_Carrera_Biologia.xlsx
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="J2" s="5" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="J3" s="5">
-        <f>COUNTIF(B6:B43, "SI")</f>
+        <f>COUNTIF(B6:B56, "SI")</f>
         <v/>
       </c>
     </row>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="J4" s="5">
-        <f>COUNTIF(C6:C43, "SI")</f>
+        <f>COUNTIF(C6:C56, "SI")</f>
         <v/>
       </c>
     </row>
@@ -667,14 +667,14 @@
         </is>
       </c>
       <c r="J5" s="5">
-        <f>COUNTIF(F6:F43, "ADEUDA FINAL")</f>
+        <f>COUNTIF(F6:F56, "ADEUDA FINAL")</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Introducción a la Biología y Sistemas Vivientes</t>
+          <t>Matemática</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
@@ -710,14 +710,14 @@
         </is>
       </c>
       <c r="J6" s="12">
-        <f>COUNTIF(B6:B43, "SI")/34</f>
+        <f>COUNTIF(B6:B56, "SI")/47</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Biología Celular y Molecular</t>
+          <t>Física</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
@@ -753,14 +753,14 @@
         </is>
       </c>
       <c r="J7" s="12">
-        <f>COUNTIF(C6:C43, "SI")/34</f>
+        <f>COUNTIF(C6:C56, "SI")/47</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Diversidad Vegetal I</t>
+          <t>Química</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -794,7 +794,7 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Química General e Inorgánica</t>
+          <t>Introducción a los sistemas vivientes</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
@@ -833,7 +833,7 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Matemática y Estadística Aplicada</t>
+          <t>Psicología educacional</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
@@ -872,7 +872,7 @@
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Pedagogía</t>
+          <t>PsicologÍa del desarrollo y del aprendizaje</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -911,7 +911,7 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Lectura, Escritura y Oralidad I (LEO 1)</t>
+          <t>Leo</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -948,37 +948,10 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Trabajo de Campo I</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>1° Año</t>
-        </is>
-      </c>
-      <c r="E13" s="10">
-        <f>IF(B13="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F13" s="10">
-        <f>IF(C13="SI", "APROBADO", IF(B13="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G13" s="11">
-        <f>IF(C13="SI", "🟢 Aprobada", IF(B13="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>📌 2° AÑO</t>
+        </is>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
@@ -987,10 +960,37 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>📌 2° AÑO</t>
-        </is>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Biología de los animales 1</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>2° Año</t>
+        </is>
+      </c>
+      <c r="E14" s="10">
+        <f>IF(B14="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F14" s="10">
+        <f>IF(C14="SI", "APROBADO", IF(B14="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G14" s="11">
+        <f>IF(C14="SI", "🟢 Aprobada", IF(B14="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
@@ -1001,7 +1001,7 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Diversidad Vegetal II</t>
+          <t>Biología de las plantas 1</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
@@ -1040,7 +1040,7 @@
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Diversidad Animal I (Invertebrados)</t>
+          <t>Biología molecular y celular</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
@@ -1074,7 +1074,7 @@
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Anatomía y Fisiología Humana</t>
+          <t>Ciencias de la tierra</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
@@ -1108,7 +1108,7 @@
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Química Orgánica y Biológica</t>
+          <t>Física biológica</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
@@ -1142,7 +1142,7 @@
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Didáctica General</t>
+          <t>Química biológica</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
@@ -1176,7 +1176,7 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Psicología Educacional</t>
+          <t>Pedagogía</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -1210,7 +1210,7 @@
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Sujetos de la Educación</t>
+          <t>Trabajo de Campo I</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
@@ -1244,7 +1244,7 @@
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>Trabajo de Campo II</t>
+          <t>DDHH, sociedad y estado</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
@@ -1275,17 +1275,44 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>📌 3° AÑO</t>
-        </is>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Taller de lengua extranjera</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>2° Año</t>
+        </is>
+      </c>
+      <c r="E23" s="10">
+        <f>IF(B23="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F23" s="10">
+        <f>IF(C23="SI", "APROBADO", IF(B23="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G23" s="11">
+        <f>IF(C23="SI", "🟢 Aprobada", IF(B23="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>Diversidad Animal II (Vertebrados)</t>
+          <t>Taller de actualización en didacticas especificas</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
@@ -1300,7 +1327,7 @@
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>3° Año</t>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E24" s="10">
@@ -1319,7 +1346,7 @@
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Genética General y Molecular</t>
+          <t>Taller de actualización disciplinar y su didactica</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
@@ -1334,7 +1361,7 @@
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>3° Año</t>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E25" s="10">
@@ -1353,7 +1380,7 @@
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>Ecología General y de Poblaciones</t>
+          <t>Nuevas tecnologias</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
@@ -1368,7 +1395,7 @@
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>3° Año</t>
+          <t>2° Año</t>
         </is>
       </c>
       <c r="E26" s="10">
@@ -1384,44 +1411,17 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>Didáctica de la Biología I</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>3° Año</t>
-        </is>
-      </c>
-      <c r="E27" s="10">
-        <f>IF(B27="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F27" s="10">
-        <f>IF(C27="SI", "APROBADO", IF(B27="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G27" s="11">
-        <f>IF(C27="SI", "🟢 Aprobada", IF(B27="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>📌 3° AÑO</t>
+        </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>Ciencias de la Tierra y Dinámica Terrestre</t>
+          <t>Genética clasica, molecular y poblacional</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
@@ -1455,7 +1455,7 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Historia Social de la Educación</t>
+          <t>Biología de las plantas 2</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
@@ -1489,7 +1489,7 @@
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>Derechos Humanos, Sociedad y Estado</t>
+          <t>Biología humana 1</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
@@ -1523,7 +1523,7 @@
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Construcción de la Práctica Docente I</t>
+          <t>Biodiversidad de las plantas</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -1554,17 +1554,44 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>📌 4° AÑO</t>
-        </is>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Biología de los animales 2</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>3° Año</t>
+        </is>
+      </c>
+      <c r="E32" s="10">
+        <f>IF(B32="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F32" s="10">
+        <f>IF(C32="SI", "APROBADO", IF(B32="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G32" s="11">
+        <f>IF(C32="SI", "🟢 Aprobada", IF(B32="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Evolución y Paleontología</t>
+          <t>Didactica general</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
@@ -1579,7 +1606,7 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>4° Año</t>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E33" s="10">
@@ -1598,7 +1625,7 @@
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>Fisiología y Morfología Comparada</t>
+          <t>Filosofía</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
@@ -1613,7 +1640,7 @@
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>4° Año</t>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E34" s="10">
@@ -1632,7 +1659,7 @@
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>Educación para la Salud y el Ambiente</t>
+          <t>Trabajod de campo 2</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
@@ -1647,7 +1674,7 @@
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>4° Año</t>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E35" s="10">
@@ -1666,7 +1693,7 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>Didáctica de la Biología II</t>
+          <t>La experimentación en biología y su didactica</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
@@ -1681,7 +1708,7 @@
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>4° Año</t>
+          <t>3° Año</t>
         </is>
       </c>
       <c r="E36" s="10">
@@ -1697,44 +1724,17 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>Educación Sexual Integral (ESI)</t>
-        </is>
-      </c>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D37" s="10" t="inlineStr">
-        <is>
-          <t>4° Año</t>
-        </is>
-      </c>
-      <c r="E37" s="10">
-        <f>IF(B37="SI", "REGULAR", "PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F37" s="10">
-        <f>IF(C37="SI", "APROBADO", IF(B37="SI", "ADEUDA FINAL", "ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G37" s="11">
-        <f>IF(C37="SI", "🟢 Aprobada", IF(B37="SI", "🟡 Regular", "🟣 Pendiente"))</f>
-        <v/>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>📌 4° AÑO</t>
+        </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>Ética y Trabajo Docente</t>
+          <t>Biología de los microorganimos, las algas y los hongos</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
@@ -1768,7 +1768,7 @@
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>Residencia y Construcción de la Práctica Docente II</t>
+          <t>Biología de los animales 3</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
@@ -1799,17 +1799,44 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>📌 TRAMO SUPERIOR / SEMINARIOS</t>
-        </is>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>Biología humana 2</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>4° Año</t>
+        </is>
+      </c>
+      <c r="E40" s="10">
+        <f>IF(B40="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F40" s="10">
+        <f>IF(C40="SI", "APROBADO", IF(B40="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G40" s="11">
+        <f>IF(C40="SI", "🟢 Aprobada", IF(B40="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>Seminario de Biotecnología y Sociedad</t>
+          <t>Dinamica terrestre</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
@@ -1824,7 +1851,7 @@
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>Tramo Superior / Seminarios</t>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E41" s="10">
@@ -1843,7 +1870,7 @@
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>Seminario de Epistemología de la Biología</t>
+          <t>Historia. filosofia y sociologia de la biología</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
@@ -1858,7 +1885,7 @@
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>Tramo Superior / Seminarios</t>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E42" s="10">
@@ -1877,7 +1904,7 @@
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>Taller de Investigación en Ciencias Naturales</t>
+          <t>Construcción practica docente 1 para el nivel medio</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
@@ -1892,7 +1919,7 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>Tramo Superior / Seminarios</t>
+          <t>4° Año</t>
         </is>
       </c>
       <c r="E43" s="10">
@@ -1908,26 +1935,441 @@
         <v/>
       </c>
     </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>Taller de educación no formal</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>4° Año</t>
+        </is>
+      </c>
+      <c r="E44" s="10">
+        <f>IF(B44="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F44" s="10">
+        <f>IF(C44="SI", "APROBADO", IF(B44="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G44" s="11">
+        <f>IF(C44="SI", "🟢 Aprobada", IF(B44="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>El lenguaje de la biología y su didactica</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>4° Año</t>
+        </is>
+      </c>
+      <c r="E45" s="10">
+        <f>IF(B45="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F45" s="10">
+        <f>IF(C45="SI", "APROBADO", IF(B45="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G45" s="11">
+        <f>IF(C45="SI", "🟢 Aprobada", IF(B45="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>Historia de la educación Argentina</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>4° Año</t>
+        </is>
+      </c>
+      <c r="E46" s="10">
+        <f>IF(B46="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F46" s="10">
+        <f>IF(C46="SI", "APROBADO", IF(B46="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G46" s="11">
+        <f>IF(C46="SI", "🟢 Aprobada", IF(B46="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>Ecología y etología</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>4° Año</t>
+        </is>
+      </c>
+      <c r="E47" s="10">
+        <f>IF(B47="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F47" s="10">
+        <f>IF(C47="SI", "APROBADO", IF(B47="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G47" s="11">
+        <f>IF(C47="SI", "🟢 Aprobada", IF(B47="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>📌 5° AÑO</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>Morfofisiologia comparada de los animales y ambiente</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>5° Año</t>
+        </is>
+      </c>
+      <c r="E49" s="10">
+        <f>IF(B49="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F49" s="10">
+        <f>IF(C49="SI", "APROBADO", IF(B49="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G49" s="11">
+        <f>IF(C49="SI", "🟢 Aprobada", IF(B49="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>Genetica, ambiente y sociedad</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>5° Año</t>
+        </is>
+      </c>
+      <c r="E50" s="10">
+        <f>IF(B50="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F50" s="10">
+        <f>IF(C50="SI", "APROBADO", IF(B50="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G50" s="11">
+        <f>IF(C50="SI", "🟢 Aprobada", IF(B50="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>Evolución e historia de la vida</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>5° Año</t>
+        </is>
+      </c>
+      <c r="E51" s="10">
+        <f>IF(B51="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F51" s="10">
+        <f>IF(C51="SI", "APROBADO", IF(B51="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G51" s="11">
+        <f>IF(C51="SI", "🟢 Aprobada", IF(B51="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>Construcción practica docente 2 y residencia niveles medio y superior</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>5° Año</t>
+        </is>
+      </c>
+      <c r="E52" s="10">
+        <f>IF(B52="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F52" s="10">
+        <f>IF(C52="SI", "APROBADO", IF(B52="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G52" s="11">
+        <f>IF(C52="SI", "🟢 Aprobada", IF(B52="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>Metodologia de la investigación</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>5° Año</t>
+        </is>
+      </c>
+      <c r="E53" s="10">
+        <f>IF(B53="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F53" s="10">
+        <f>IF(C53="SI", "APROBADO", IF(B53="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G53" s="11">
+        <f>IF(C53="SI", "🟢 Aprobada", IF(B53="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>Educación para la salud</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>5° Año</t>
+        </is>
+      </c>
+      <c r="E54" s="10">
+        <f>IF(B54="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F54" s="10">
+        <f>IF(C54="SI", "APROBADO", IF(B54="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G54" s="11">
+        <f>IF(C54="SI", "🟢 Aprobada", IF(B54="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>Sistema y politica educativa</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>5° Año</t>
+        </is>
+      </c>
+      <c r="E55" s="10">
+        <f>IF(B55="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F55" s="10">
+        <f>IF(C55="SI", "APROBADO", IF(B55="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G55" s="11">
+        <f>IF(C55="SI", "🟢 Aprobada", IF(B55="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t>Didactica de la educación en el ambiente y la sustentabilidad</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t>5° Año</t>
+        </is>
+      </c>
+      <c r="E56" s="10">
+        <f>IF(B56="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F56" s="10">
+        <f>IF(C56="SI", "APROBADO", IF(B56="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G56" s="11">
+        <f>IF(C56="SI", "🟢 Aprobada", IF(B56="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A32:G32"/>
-    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A13:G13"/>
     <mergeCell ref="I12:J12"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A27:G27"/>
     <mergeCell ref="I15:J15"/>
     <mergeCell ref="I10:J10"/>
     <mergeCell ref="I1:K1"/>
+    <mergeCell ref="A48:G48"/>
     <mergeCell ref="I11:J11"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="I13:J13"/>
     <mergeCell ref="I14:J14"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B6 B7 B8 B9 B10 B11 B12 B13 B15 B16 B17 B18 B19 B20 B21 B22 B24 B25 B26 B27 B28 B29 B30 B31 B33 B34 B35 B36 B37 B38 B39 B41 B42 B43 C6 C7 C8 C9 C10 C11 C12 C13 C15 C16 C17 C18 C19 C20 C21 C22 C24 C25 C26 C27 C28 C29 C30 C31 C33 C34 C35 C36 C37 C38 C39 C41 C42 C43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Opción inválida" error="Por favor, elegí 'SI' o 'NO' de la lista desplegable." type="list">
+    <dataValidation sqref="B6 B7 B8 B9 B10 B11 B12 B14 B15 B16 B17 B18 B19 B20 B21 B22 B23 B24 B25 B26 B28 B29 B30 B31 B32 B33 B34 B35 B36 B38 B39 B40 B41 B42 B43 B44 B45 B46 B47 B49 B50 B51 B52 B53 B54 B55 B56 C6 C7 C8 C9 C10 C11 C12 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C28 C29 C30 C31 C32 C33 C34 C35 C36 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C49 C50 C51 C52 C53 C54 C55 C56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Opción inválida" error="Por favor, elegí 'SI' o 'NO' de la lista desplegable." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>